<commit_message>
Changes updated on 28 Aug
</commit_message>
<xml_diff>
--- a/12608100.xlsx
+++ b/12608100.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/178e7b8b65df52d4/Desktop/CAP-776/CAP776/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="189" documentId="8_{423A2F30-43C3-4C4F-AB9B-22B4BC24882D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{64FA0484-9D7E-4DC9-8EB3-94BE98FE2479}"/>
+  <xr:revisionPtr revIDLastSave="222" documentId="8_{423A2F30-43C3-4C4F-AB9B-22B4BC24882D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BF366A04-68B1-460F-8142-F4045BF8BD6D}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="80">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -266,6 +266,15 @@
   </si>
   <si>
     <t xml:space="preserve">Feeling a little exhausted but it's fine </t>
+  </si>
+  <si>
+    <t>Feeling nice</t>
+  </si>
+  <si>
+    <t>Didn't able to do something productive due to electricity cut.</t>
+  </si>
+  <si>
+    <t>Happy to try a new recipe.</t>
   </si>
 </sst>
 </file>
@@ -546,6 +555,10 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -1738,73 +1751,139 @@
       <c r="A21" s="8">
         <v>46260</v>
       </c>
-      <c r="B21" s="13"/>
-      <c r="C21" s="13"/>
-      <c r="D21" s="13"/>
-      <c r="E21" s="13"/>
-      <c r="F21" s="13"/>
-      <c r="G21" s="13"/>
-      <c r="H21" s="13"/>
-      <c r="I21" s="14" t="str">
+      <c r="B21" s="13">
+        <v>350</v>
+      </c>
+      <c r="C21" s="13">
+        <v>30</v>
+      </c>
+      <c r="D21" s="13">
+        <v>60</v>
+      </c>
+      <c r="E21" s="13">
+        <v>120</v>
+      </c>
+      <c r="F21" s="13">
+        <v>400</v>
+      </c>
+      <c r="G21" s="13">
+        <v>4</v>
+      </c>
+      <c r="H21" s="13">
+        <v>120</v>
+      </c>
+      <c r="I21" s="14">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J21" s="14" t="str">
+        <v>1080</v>
+      </c>
+      <c r="J21" s="14">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K21" s="15"/>
-      <c r="L21" s="15"/>
-      <c r="M21" s="15"/>
-      <c r="N21" s="16"/>
-    </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.3">
+        <v>360</v>
+      </c>
+      <c r="K21" s="15" t="s">
+        <v>49</v>
+      </c>
+      <c r="L21" s="15" t="s">
+        <v>57</v>
+      </c>
+      <c r="M21" s="15" t="s">
+        <v>51</v>
+      </c>
+      <c r="N21" s="16" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="22" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A22" s="8">
         <v>46261</v>
       </c>
-      <c r="B22" s="13"/>
-      <c r="C22" s="13"/>
-      <c r="D22" s="13"/>
-      <c r="E22" s="13"/>
-      <c r="F22" s="13"/>
-      <c r="G22" s="13"/>
-      <c r="H22" s="13"/>
-      <c r="I22" s="14" t="str">
+      <c r="B22" s="13">
+        <v>420</v>
+      </c>
+      <c r="C22" s="13">
+        <v>40</v>
+      </c>
+      <c r="D22" s="13">
+        <v>30</v>
+      </c>
+      <c r="E22" s="13">
+        <v>30</v>
+      </c>
+      <c r="F22" s="13">
+        <v>350</v>
+      </c>
+      <c r="G22" s="13">
+        <v>7</v>
+      </c>
+      <c r="H22" s="13">
+        <v>60</v>
+      </c>
+      <c r="I22" s="14">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J22" s="14" t="str">
+        <v>930</v>
+      </c>
+      <c r="J22" s="14">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K22" s="15"/>
-      <c r="L22" s="15"/>
-      <c r="M22" s="15"/>
-      <c r="N22" s="16"/>
+        <v>510</v>
+      </c>
+      <c r="K22" s="15" t="s">
+        <v>60</v>
+      </c>
+      <c r="L22" s="15" t="s">
+        <v>50</v>
+      </c>
+      <c r="M22" s="15" t="s">
+        <v>55</v>
+      </c>
+      <c r="N22" s="16" t="s">
+        <v>78</v>
+      </c>
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A23" s="8">
         <v>46262</v>
       </c>
-      <c r="B23" s="13"/>
-      <c r="C23" s="13"/>
-      <c r="D23" s="13"/>
-      <c r="E23" s="13"/>
-      <c r="F23" s="13"/>
-      <c r="G23" s="13"/>
-      <c r="H23" s="13"/>
-      <c r="I23" s="14" t="str">
+      <c r="B23" s="13">
+        <v>480</v>
+      </c>
+      <c r="C23" s="13">
+        <v>20</v>
+      </c>
+      <c r="D23" s="13">
+        <v>120</v>
+      </c>
+      <c r="E23" s="13">
+        <v>60</v>
+      </c>
+      <c r="F23" s="13">
+        <v>100</v>
+      </c>
+      <c r="G23" s="13">
+        <v>2</v>
+      </c>
+      <c r="H23" s="13">
+        <v>180</v>
+      </c>
+      <c r="I23" s="14">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J23" s="14" t="str">
+        <v>960</v>
+      </c>
+      <c r="J23" s="14">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K23" s="15"/>
-      <c r="L23" s="15"/>
-      <c r="M23" s="15"/>
-      <c r="N23" s="16"/>
+        <v>480</v>
+      </c>
+      <c r="K23" s="15" t="s">
+        <v>60</v>
+      </c>
+      <c r="L23" s="15" t="s">
+        <v>50</v>
+      </c>
+      <c r="M23" s="15" t="s">
+        <v>51</v>
+      </c>
+      <c r="N23" s="16" t="s">
+        <v>79</v>
+      </c>
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A24" s="8">

</xml_diff>

<commit_message>
Updated on 30 August
</commit_message>
<xml_diff>
--- a/12608100.xlsx
+++ b/12608100.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/178e7b8b65df52d4/Desktop/CAP-776/CAP776/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="222" documentId="8_{423A2F30-43C3-4C4F-AB9B-22B4BC24882D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BF366A04-68B1-460F-8142-F4045BF8BD6D}"/>
+  <xr:revisionPtr revIDLastSave="244" documentId="8_{423A2F30-43C3-4C4F-AB9B-22B4BC24882D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1DEE4255-A10E-4506-AE71-A188246DA6B9}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="82">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -275,6 +275,12 @@
   </si>
   <si>
     <t>Happy to try a new recipe.</t>
+  </si>
+  <si>
+    <t>Weekends feels boring sometimes</t>
+  </si>
+  <si>
+    <t>Again the same classes from tommorow</t>
   </si>
 </sst>
 </file>
@@ -1885,53 +1891,97 @@
         <v>79</v>
       </c>
     </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A24" s="8">
         <v>46263</v>
       </c>
-      <c r="B24" s="13"/>
-      <c r="C24" s="13"/>
-      <c r="D24" s="13"/>
-      <c r="E24" s="13"/>
-      <c r="F24" s="13"/>
-      <c r="G24" s="13"/>
-      <c r="H24" s="13"/>
-      <c r="I24" s="14" t="str">
+      <c r="B24" s="13">
+        <v>540</v>
+      </c>
+      <c r="C24" s="13">
+        <v>20</v>
+      </c>
+      <c r="D24" s="13">
+        <v>180</v>
+      </c>
+      <c r="E24" s="13">
+        <v>0</v>
+      </c>
+      <c r="F24" s="13">
+        <v>0</v>
+      </c>
+      <c r="G24" s="13">
+        <v>0</v>
+      </c>
+      <c r="H24" s="13">
+        <v>120</v>
+      </c>
+      <c r="I24" s="14">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J24" s="14" t="str">
+        <v>860</v>
+      </c>
+      <c r="J24" s="14">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K24" s="15"/>
-      <c r="L24" s="15"/>
-      <c r="M24" s="15"/>
-      <c r="N24" s="16"/>
-    </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.3">
+        <v>580</v>
+      </c>
+      <c r="K24" s="15" t="s">
+        <v>60</v>
+      </c>
+      <c r="L24" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="M24" s="15" t="s">
+        <v>51</v>
+      </c>
+      <c r="N24" s="16" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="25" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A25" s="8">
         <v>46264</v>
       </c>
-      <c r="B25" s="13"/>
-      <c r="C25" s="13"/>
-      <c r="D25" s="13"/>
-      <c r="E25" s="13"/>
-      <c r="F25" s="13"/>
-      <c r="G25" s="13"/>
-      <c r="H25" s="13"/>
-      <c r="I25" s="14" t="str">
+      <c r="B25" s="13">
+        <v>600</v>
+      </c>
+      <c r="C25" s="13">
+        <v>20</v>
+      </c>
+      <c r="D25" s="13">
+        <v>120</v>
+      </c>
+      <c r="E25" s="13">
+        <v>120</v>
+      </c>
+      <c r="F25" s="13">
+        <v>0</v>
+      </c>
+      <c r="G25" s="13">
+        <v>0</v>
+      </c>
+      <c r="H25" s="13">
+        <v>180</v>
+      </c>
+      <c r="I25" s="14">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J25" s="14" t="str">
+        <v>1040</v>
+      </c>
+      <c r="J25" s="14">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K25" s="15"/>
-      <c r="L25" s="15"/>
-      <c r="M25" s="15"/>
-      <c r="N25" s="16"/>
+        <v>400</v>
+      </c>
+      <c r="K25" s="15" t="s">
+        <v>49</v>
+      </c>
+      <c r="L25" s="15" t="s">
+        <v>57</v>
+      </c>
+      <c r="M25" s="15" t="s">
+        <v>51</v>
+      </c>
+      <c r="N25" s="16" t="s">
+        <v>81</v>
+      </c>
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A26" s="8">

</xml_diff>

<commit_message>
Updated on 9 sept
</commit_message>
<xml_diff>
--- a/12608100.xlsx
+++ b/12608100.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/178e7b8b65df52d4/Desktop/CAP-776/CAP776/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="312" documentId="8_{423A2F30-43C3-4C4F-AB9B-22B4BC24882D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A83119D9-2270-4046-A8BB-F79FFDFE3692}"/>
+  <xr:revisionPtr revIDLastSave="348" documentId="8_{423A2F30-43C3-4C4F-AB9B-22B4BC24882D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9A285848-CEBF-490D-A596-6369E561FB66}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="89">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -293,6 +293,15 @@
   </si>
   <si>
     <t>Missed classes for the first time in this semester</t>
+  </si>
+  <si>
+    <t>Too lazy</t>
+  </si>
+  <si>
+    <t>Preparing for CA</t>
+  </si>
+  <si>
+    <t>Today 2 CAs</t>
   </si>
 </sst>
 </file>
@@ -2229,73 +2238,139 @@
       <c r="A31" s="8">
         <v>46270</v>
       </c>
-      <c r="B31" s="13"/>
-      <c r="C31" s="13"/>
-      <c r="D31" s="13"/>
-      <c r="E31" s="13"/>
-      <c r="F31" s="13"/>
-      <c r="G31" s="13"/>
-      <c r="H31" s="13"/>
-      <c r="I31" s="14" t="str">
+      <c r="B31" s="13">
+        <v>540</v>
+      </c>
+      <c r="C31" s="13">
+        <v>0</v>
+      </c>
+      <c r="D31" s="13">
+        <v>120</v>
+      </c>
+      <c r="E31" s="13">
+        <v>60</v>
+      </c>
+      <c r="F31" s="13">
+        <v>0</v>
+      </c>
+      <c r="G31" s="13">
+        <v>0</v>
+      </c>
+      <c r="H31" s="13">
+        <v>120</v>
+      </c>
+      <c r="I31" s="14">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J31" s="14" t="str">
+        <v>840</v>
+      </c>
+      <c r="J31" s="14">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K31" s="15"/>
-      <c r="L31" s="15"/>
-      <c r="M31" s="15"/>
-      <c r="N31" s="16"/>
+        <v>600</v>
+      </c>
+      <c r="K31" s="15" t="s">
+        <v>49</v>
+      </c>
+      <c r="L31" s="15" t="s">
+        <v>57</v>
+      </c>
+      <c r="M31" s="15" t="s">
+        <v>56</v>
+      </c>
+      <c r="N31" s="16" t="s">
+        <v>86</v>
+      </c>
     </row>
     <row r="32" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A32" s="8">
         <v>46271</v>
       </c>
-      <c r="B32" s="13"/>
-      <c r="C32" s="13"/>
-      <c r="D32" s="13"/>
-      <c r="E32" s="13"/>
-      <c r="F32" s="13"/>
-      <c r="G32" s="13"/>
-      <c r="H32" s="13"/>
-      <c r="I32" s="14" t="str">
+      <c r="B32" s="13">
+        <v>540</v>
+      </c>
+      <c r="C32" s="13">
+        <v>20</v>
+      </c>
+      <c r="D32" s="13">
+        <v>180</v>
+      </c>
+      <c r="E32" s="13">
+        <v>30</v>
+      </c>
+      <c r="F32" s="13">
+        <v>0</v>
+      </c>
+      <c r="G32" s="13">
+        <v>0</v>
+      </c>
+      <c r="H32" s="13">
+        <v>120</v>
+      </c>
+      <c r="I32" s="14">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J32" s="14" t="str">
+        <v>890</v>
+      </c>
+      <c r="J32" s="14">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K32" s="15"/>
-      <c r="L32" s="15"/>
-      <c r="M32" s="15"/>
-      <c r="N32" s="16"/>
+        <v>550</v>
+      </c>
+      <c r="K32" s="15" t="s">
+        <v>60</v>
+      </c>
+      <c r="L32" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="M32" s="15" t="s">
+        <v>51</v>
+      </c>
+      <c r="N32" s="16" t="s">
+        <v>87</v>
+      </c>
     </row>
     <row r="33" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A33" s="8">
         <v>46272</v>
       </c>
-      <c r="B33" s="13"/>
-      <c r="C33" s="13"/>
-      <c r="D33" s="13"/>
-      <c r="E33" s="13"/>
-      <c r="F33" s="13"/>
-      <c r="G33" s="13"/>
-      <c r="H33" s="13"/>
-      <c r="I33" s="14" t="str">
+      <c r="B33" s="13">
+        <v>420</v>
+      </c>
+      <c r="C33" s="13">
+        <v>30</v>
+      </c>
+      <c r="D33" s="13">
+        <v>210</v>
+      </c>
+      <c r="E33" s="13">
+        <v>30</v>
+      </c>
+      <c r="F33" s="13">
+        <v>200</v>
+      </c>
+      <c r="G33" s="13">
+        <v>4</v>
+      </c>
+      <c r="H33" s="13">
+        <v>90</v>
+      </c>
+      <c r="I33" s="14">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J33" s="14" t="str">
+        <v>980</v>
+      </c>
+      <c r="J33" s="14">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K33" s="15"/>
-      <c r="L33" s="15"/>
-      <c r="M33" s="15"/>
-      <c r="N33" s="16"/>
+        <v>460</v>
+      </c>
+      <c r="K33" s="15" t="s">
+        <v>49</v>
+      </c>
+      <c r="L33" s="15" t="s">
+        <v>50</v>
+      </c>
+      <c r="M33" s="15" t="s">
+        <v>51</v>
+      </c>
+      <c r="N33" s="16" t="s">
+        <v>88</v>
+      </c>
     </row>
     <row r="34" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A34" s="8">

</xml_diff>